<commit_message>
feat: mettre à jour le lien de téléchargement du tableau de synthèse E5 et ajouter un fichier temporaire
</commit_message>
<xml_diff>
--- a/documents/Tableau_synthese_E5.xlsx
+++ b/documents/Tableau_synthese_E5.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\BTS\2025\CIRCULAIRES NATIONALES\SIO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Portfolio\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0B016ED-F93A-4E72-B6C7-69DD0949F443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11250"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
@@ -106,9 +107,6 @@
     <t xml:space="preserve">N° candidat : </t>
   </si>
   <si>
-    <t xml:space="preserve">NOM et prénom : </t>
-  </si>
-  <si>
     <t>Période (sous la forme du JJ/MM/AA au JJ/MM/AA)</t>
   </si>
   <si>
@@ -118,16 +116,19 @@
     <t>Réalisations en milieu professionnel en cours de seconde année</t>
   </si>
   <si>
-    <t>Adresse URL du portfolio :</t>
-  </si>
-  <si>
     <t>SESSION 2025</t>
+  </si>
+  <si>
+    <t>NOM et prénom : SANJIVY Romain</t>
+  </si>
+  <si>
+    <t>Adresse URL du portfolio : https://portfolio-romain.testoxylog.fr/</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
@@ -593,7 +594,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -601,13 +602,13 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -616,28 +617,22 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -646,13 +641,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -661,31 +650,55 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -697,10 +710,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -712,33 +725,9 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Euro" xfId="1"/>
+    <cellStyle name="Euro" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -755,9 +744,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -795,9 +784,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -832,7 +821,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -867,7 +856,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1040,99 +1029,99 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:AQ81"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="70.42578125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.85546875" style="1" customWidth="1"/>
-    <col min="3" max="8" width="18.7109375" style="1" customWidth="1"/>
-    <col min="9" max="43" width="11.42578125" customWidth="1"/>
-    <col min="44" max="16384" width="10.85546875" style="1"/>
+    <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" style="1" customWidth="1"/>
+    <col min="3" max="8" width="18.6640625" style="1" customWidth="1"/>
+    <col min="9" max="43" width="11.44140625" customWidth="1"/>
+    <col min="44" max="16384" width="10.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="28" t="s">
+    <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28" t="s">
-        <v>26</v>
-      </c>
-      <c r="H1" s="28"/>
-    </row>
-    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="28" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="H1" s="22"/>
+    </row>
+    <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="28"/>
-      <c r="C2" s="28"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="28"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
-      <c r="H2" s="28"/>
-    </row>
-    <row r="3" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="40" t="s">
-        <v>21</v>
-      </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="42"/>
-      <c r="F3" s="46" t="s">
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+    </row>
+    <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="41"/>
-      <c r="H3" s="47"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="30"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
-    <row r="4" spans="1:43" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="43" t="s">
+    <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="44"/>
-      <c r="C4" s="44"/>
-      <c r="D4" s="44"/>
-      <c r="E4" s="45"/>
-      <c r="F4" s="16" t="s">
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="27"/>
+      <c r="E4" s="28"/>
+      <c r="F4" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="G4" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="H4" s="21" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:43" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="37" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="38"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="38"/>
-      <c r="G5" s="38"/>
-      <c r="H5" s="39"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="26" t="s">
+    <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="43"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="35" t="s">
-        <v>22</v>
+      <c r="B6" s="39" t="s">
+        <v>21</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>0</v>
@@ -1153,9 +1142,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="27"/>
-      <c r="B7" s="36"/>
+    <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="32"/>
+      <c r="B7" s="40"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1210,17 +1199,17 @@
       <c r="AP7"/>
       <c r="AQ7"/>
     </row>
-    <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A8" s="29" t="s">
+    <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A8" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="30"/>
-      <c r="C8" s="30"/>
-      <c r="D8" s="30"/>
-      <c r="E8" s="30"/>
-      <c r="F8" s="30"/>
-      <c r="G8" s="30"/>
-      <c r="H8" s="31"/>
+      <c r="B8" s="34"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="34"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="34"/>
+      <c r="G8" s="34"/>
+      <c r="H8" s="35"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1257,15 +1246,15 @@
       <c r="AP8"/>
       <c r="AQ8"/>
     </row>
-    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="12"/>
+    <row r="9" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="11"/>
       <c r="B9" s="10"/>
-      <c r="C9" s="18"/>
-      <c r="D9" s="19"/>
-      <c r="E9" s="19"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="20"/>
+      <c r="C9" s="16"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="17"/>
+      <c r="F9" s="17"/>
+      <c r="G9" s="17"/>
+      <c r="H9" s="18"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1302,15 +1291,15 @@
       <c r="AP9"/>
       <c r="AQ9"/>
     </row>
-    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="12"/>
+    <row r="10" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="11"/>
       <c r="B10" s="10"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="20"/>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
+      <c r="G10" s="17"/>
+      <c r="H10" s="18"/>
       <c r="I10"/>
       <c r="J10"/>
       <c r="K10"/>
@@ -1347,15 +1336,15 @@
       <c r="AP10"/>
       <c r="AQ10"/>
     </row>
-    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="12"/>
+    <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="11"/>
       <c r="B11" s="10"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="20"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
+      <c r="G11" s="17"/>
+      <c r="H11" s="18"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1392,15 +1381,15 @@
       <c r="AP11"/>
       <c r="AQ11"/>
     </row>
-    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="12"/>
+    <row r="12" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="11"/>
       <c r="B12" s="10"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="20"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="17"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
+      <c r="G12" s="17"/>
+      <c r="H12" s="18"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1437,15 +1426,15 @@
       <c r="AP12"/>
       <c r="AQ12"/>
     </row>
-    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="12"/>
+    <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="11"/>
       <c r="B13" s="10"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="20"/>
+      <c r="C13" s="17"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
+      <c r="G13" s="17"/>
+      <c r="H13" s="18"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1482,15 +1471,15 @@
       <c r="AP13"/>
       <c r="AQ13"/>
     </row>
-    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="12"/>
+    <row r="14" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="11"/>
       <c r="B14" s="10"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="20"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
+      <c r="G14" s="17"/>
+      <c r="H14" s="18"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1527,15 +1516,15 @@
       <c r="AP14"/>
       <c r="AQ14"/>
     </row>
-    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="12"/>
+    <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="11"/>
       <c r="B15" s="10"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="20"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
+      <c r="G15" s="17"/>
+      <c r="H15" s="18"/>
       <c r="I15"/>
       <c r="J15"/>
       <c r="K15"/>
@@ -1572,15 +1561,15 @@
       <c r="AP15"/>
       <c r="AQ15"/>
     </row>
-    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="12"/>
+    <row r="16" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="11"/>
       <c r="B16" s="10"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="20"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="18"/>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1617,15 +1606,15 @@
       <c r="AP16"/>
       <c r="AQ16"/>
     </row>
-    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="12"/>
+    <row r="17" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="11"/>
       <c r="B17" s="10"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="20"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
+      <c r="G17" s="17"/>
+      <c r="H17" s="18"/>
       <c r="I17"/>
       <c r="J17"/>
       <c r="K17"/>
@@ -1662,15 +1651,15 @@
       <c r="AP17"/>
       <c r="AQ17"/>
     </row>
-    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="12"/>
+    <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="11"/>
       <c r="B18" s="10"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="20"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="18"/>
       <c r="I18"/>
       <c r="J18"/>
       <c r="K18"/>
@@ -1707,17 +1696,17 @@
       <c r="AP18"/>
       <c r="AQ18"/>
     </row>
-    <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A19" s="32" t="s">
-        <v>23</v>
-      </c>
-      <c r="B19" s="33"/>
-      <c r="C19" s="33"/>
-      <c r="D19" s="33"/>
-      <c r="E19" s="33"/>
-      <c r="F19" s="33"/>
-      <c r="G19" s="33"/>
-      <c r="H19" s="34"/>
+    <row r="19" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A19" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="37"/>
+      <c r="C19" s="37"/>
+      <c r="D19" s="37"/>
+      <c r="E19" s="37"/>
+      <c r="F19" s="37"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="38"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -1754,15 +1743,15 @@
       <c r="AP19"/>
       <c r="AQ19"/>
     </row>
-    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="12"/>
+    <row r="20" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="11"/>
       <c r="B20" s="10"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="20"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="18"/>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>
@@ -1799,15 +1788,15 @@
       <c r="AP20"/>
       <c r="AQ20"/>
     </row>
-    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="12"/>
+    <row r="21" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="11"/>
       <c r="B21" s="10"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="20"/>
+      <c r="C21" s="17"/>
+      <c r="D21" s="17"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
+      <c r="G21" s="17"/>
+      <c r="H21" s="18"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -1844,15 +1833,15 @@
       <c r="AP21"/>
       <c r="AQ21"/>
     </row>
-    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="12"/>
+    <row r="22" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="11"/>
       <c r="B22" s="10"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="20"/>
+      <c r="C22" s="17"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
+      <c r="G22" s="17"/>
+      <c r="H22" s="18"/>
       <c r="I22"/>
       <c r="J22"/>
       <c r="K22"/>
@@ -1889,15 +1878,15 @@
       <c r="AP22"/>
       <c r="AQ22"/>
     </row>
-    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="12"/>
+    <row r="23" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="11"/>
       <c r="B23" s="10"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="20"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="18"/>
       <c r="I23"/>
       <c r="J23"/>
       <c r="K23"/>
@@ -1934,15 +1923,15 @@
       <c r="AP23"/>
       <c r="AQ23"/>
     </row>
-    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="12"/>
+    <row r="24" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="11"/>
       <c r="B24" s="10"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="20"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="18"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -1979,15 +1968,15 @@
       <c r="AP24"/>
       <c r="AQ24"/>
     </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="12"/>
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="11"/>
       <c r="B25" s="10"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="20"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="18"/>
       <c r="I25"/>
       <c r="J25"/>
       <c r="K25"/>
@@ -2024,15 +2013,15 @@
       <c r="AP25"/>
       <c r="AQ25"/>
     </row>
-    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="12"/>
+    <row r="26" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="11"/>
       <c r="B26" s="10"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="20"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
+      <c r="G26" s="17"/>
+      <c r="H26" s="18"/>
       <c r="I26"/>
       <c r="J26"/>
       <c r="K26"/>
@@ -2069,17 +2058,17 @@
       <c r="AP26"/>
       <c r="AQ26"/>
     </row>
-    <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.2">
-      <c r="A27" s="32" t="s">
-        <v>24</v>
-      </c>
-      <c r="B27" s="33"/>
-      <c r="C27" s="33"/>
-      <c r="D27" s="33"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="33"/>
-      <c r="H27" s="34"/>
+    <row r="27" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A27" s="36" t="s">
+        <v>23</v>
+      </c>
+      <c r="B27" s="37"/>
+      <c r="C27" s="37"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="38"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2116,15 +2105,15 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="12"/>
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="11"/>
       <c r="B28" s="10"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="20"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="18"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2161,15 +2150,15 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="12"/>
+    <row r="29" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="11"/>
       <c r="B29" s="10"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="19"/>
-      <c r="H29" s="20"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="18"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2206,15 +2195,15 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="12"/>
+    <row r="30" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="11"/>
       <c r="B30" s="10"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="20"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="17"/>
+      <c r="H30" s="18"/>
       <c r="I30"/>
       <c r="J30"/>
       <c r="K30"/>
@@ -2251,15 +2240,15 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="12"/>
+    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="11"/>
       <c r="B31" s="10"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="20"/>
+      <c r="C31" s="17"/>
+      <c r="D31" s="17"/>
+      <c r="E31" s="17"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="17"/>
+      <c r="H31" s="18"/>
       <c r="I31"/>
       <c r="J31"/>
       <c r="K31"/>
@@ -2296,15 +2285,15 @@
       <c r="AP31"/>
       <c r="AQ31"/>
     </row>
-    <row r="32" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="12"/>
+    <row r="32" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="11"/>
       <c r="B32" s="10"/>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="20"/>
+      <c r="C32" s="17"/>
+      <c r="D32" s="17"/>
+      <c r="E32" s="17"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="17"/>
+      <c r="H32" s="18"/>
       <c r="I32"/>
       <c r="J32"/>
       <c r="K32"/>
@@ -2341,15 +2330,15 @@
       <c r="AP32"/>
       <c r="AQ32"/>
     </row>
-    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="13"/>
-      <c r="B33" s="11"/>
-      <c r="C33" s="21"/>
-      <c r="D33" s="21"/>
-      <c r="E33" s="21"/>
-      <c r="F33" s="21"/>
-      <c r="G33" s="21"/>
-      <c r="H33" s="22"/>
+    <row r="33" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="11"/>
+      <c r="B33" s="10"/>
+      <c r="C33" s="17"/>
+      <c r="D33" s="17"/>
+      <c r="E33" s="17"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="17"/>
+      <c r="H33" s="18"/>
       <c r="I33"/>
       <c r="J33"/>
       <c r="K33"/>
@@ -2386,15 +2375,15 @@
       <c r="AP33"/>
       <c r="AQ33"/>
     </row>
-    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="14"/>
-      <c r="B34" s="15"/>
-      <c r="C34" s="23"/>
-      <c r="D34" s="23"/>
-      <c r="E34" s="23"/>
-      <c r="F34" s="23"/>
-      <c r="G34" s="23"/>
-      <c r="H34" s="24"/>
+    <row r="34" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="12"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="19"/>
+      <c r="D34" s="19"/>
+      <c r="E34" s="19"/>
+      <c r="F34" s="19"/>
+      <c r="G34" s="19"/>
+      <c r="H34" s="20"/>
       <c r="I34"/>
       <c r="J34"/>
       <c r="K34"/>
@@ -2431,7 +2420,7 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
       <c r="A35" s="5"/>
       <c r="B35" s="3"/>
       <c r="C35" s="4"/>
@@ -2476,59 +2465,54 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="49" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="50" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="51" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="52" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="53" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="54" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="55" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="56" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="57" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="58" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="59" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="60" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="61" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="62" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="63" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="64" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="65" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="66" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="67" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="68" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="69" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="70" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="71" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="72" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="73" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="74" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="75" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="76" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="77" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="78" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="79" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="80" customFormat="1" x14ac:dyDescent="0.2"/>
-    <row r="81" customFormat="1" x14ac:dyDescent="0.2"/>
+    <row r="36" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="41" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="42" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="43" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="44" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="45" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="46" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="47" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="48" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="49" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="50" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="51" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="52" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="53" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="54" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="55" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="56" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="57" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="58" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="59" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="60" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="61" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="62" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="63" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="64" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="65" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="66" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="67" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="68" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="69" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="70" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="71" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="72" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="73" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="74" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="75" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="76" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="77" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="78" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="79" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="80" customFormat="1" x14ac:dyDescent="0.25"/>
+    <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2536,11 +2520,16 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="48" orientation="portrait"/>
+  <pageSetup paperSize="9" scale="48" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: mettre à jour le tableau de synthèse E5 et réorganiser les projets dans index.html
</commit_message>
<xml_diff>
--- a/documents/Tableau_synthese_E5.xlsx
+++ b/documents/Tableau_synthese_E5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Portfolio\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF227D61-9600-465A-AEF4-46E31B7C2D35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F881C9B3-3619-4FD8-9037-06562F2E2EC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Tableau de synthèse Épreuve E5" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$37</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tableau de synthèse Épreuve E5'!$A$1:$H$36</definedName>
   </definedNames>
   <calcPr calcId="101716"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="45">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -86,12 +86,6 @@
 ▸Développer son projet professionnel</t>
   </si>
   <si>
-    <t>▢ SISR</t>
-  </si>
-  <si>
-    <t>▢ SLAM</t>
-  </si>
-  <si>
     <t xml:space="preserve">Réalisation en cours de formation
 </t>
   </si>
@@ -113,9 +107,6 @@
     <t>Réalisations en milieu professionnel en cours de seconde année</t>
   </si>
   <si>
-    <t>SESSION 2025</t>
-  </si>
-  <si>
     <t>NOM et prénom : SANJIVY Romain</t>
   </si>
   <si>
@@ -126,6 +117,97 @@
   </si>
   <si>
     <t>X</t>
+  </si>
+  <si>
+    <r>
+      <t>Mise en place de la double authentification PASSKEY</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>participation au déploiement d’une solution d’authentification renforcée pour sécuriser l’accès aux services de l’entreprise. Accompagnement des utilisateurs dans l’activation de la solution, vérification du bon fonctionnement et assistance en cas de difficulté</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Support à la migration Windows 10 vers Windows 11</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>participation à la préparation et à l’accompagnement des utilisateurs dans le cadre de la migration des postes de travail vers Windows 11. Vérification de la compatibilité, assistance aux utilisateurs, résolution des incidents post-migration et suivi des opérations.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Réorganisation du kiosque IT</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>participation à la réorganisation du kiosque informatique afin d’améliorer la gestion des équipements, la lisibilité des ressources disponibles et l’efficacité de la prise en charge des utilisateurs.</t>
+    </r>
+  </si>
+  <si>
+    <t>01/04/2025 au 15/04/2025</t>
+  </si>
+  <si>
+    <t>2024-2026</t>
+  </si>
+  <si>
+    <t>2025-2026</t>
+  </si>
+  <si>
+    <t>02/09/2024 au 02/09/2026</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Projet RMS Ticket  : </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>développement d’une application web de gestion de tickets permettant le suivi des demandes, la gestion des incidents, des utilisateurs et des rôles. Langages utilisés : PHP, JavaScript, CSS et HTML</t>
+    </r>
   </si>
   <si>
     <r>
@@ -137,30 +219,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>développement d’une application web de musculation reliée à une base de données, avec création de comptes, authentification, gestion des rôles, programmes d’entraînement et abonnements.</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Projet RMS Ticket  : </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>développement d’une application web de gestion de tickets permettant le suivi des demandes, la gestion des incidents, des utilisateurs et des rôles.</t>
+      <t>développement d’une application web de musculation reliée à une base de données, avec création de comptes, authentification, gestion des programmes d’entraînement et abonnements. Langages utilisés : PHP, JavaScript, CSS et HTML</t>
     </r>
     <r>
       <rPr>
@@ -194,6 +253,23 @@
       </rPr>
       <t>conception et développement d’un site web portfolio permettant de présenter mon profil, mes compétences, mes projets et mon parcours professionnel. Mise en ligne du site et mise à jour des contenus.</t>
     </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Langages utilisés : JavaScript, CSS et HTML</t>
+    </r>
   </si>
   <si>
     <r>
@@ -216,84 +292,67 @@
       </rPr>
       <t>conception et développement d’un site web de présentation/location d’une maison de vacances, avec mise en forme des contenus, formulaire de contact et éventuelle gestion de données selon l’architecture retenue.</t>
     </r>
-  </si>
-  <si>
     <r>
-      <t>Mise en place de la double authentification PASSKEY</t>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
-        <b/>
-        <sz val="10"/>
+        <sz val="11"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> : </t>
+      <t>Langages utilisés : JavaScript, CSS et HTML</t>
+    </r>
+  </si>
+  <si>
+    <t>☒ SLAM</t>
+  </si>
+  <si>
+    <t>☐ SISR</t>
+  </si>
+  <si>
+    <t>SESSION 2026</t>
+  </si>
+  <si>
+    <t>02/09/2024 au …</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Déplacement sur le site de Semoy : </t>
     </r>
     <r>
       <rPr>
-        <sz val="10"/>
+        <sz val="11"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>participation au déploiement d’une solution d’authentification renforcée pour sécuriser l’accès aux services de l’entreprise. Accompagnement des utilisateurs dans l’activation de la solution, vérification du bon fonctionnement et assistance en cas de difficulté</t>
+      <t>participation au renouvellement du parc informatique sur le site, avec préparation, masterisation, installation et remplacement de postes de travail. Prise en compte de l’environnement technique local, vérification du bon fonctionnement du matériel et accompagnement des utilisateurs lors de la remise en service.</t>
     </r>
   </si>
   <si>
     <r>
-      <t>Support à la migration Windows 10 vers Windows 11</t>
+      <t xml:space="preserve">Déplacement sur le site de Calais : </t>
     </r>
     <r>
       <rPr>
-        <b/>
-        <sz val="10"/>
+        <sz val="11"/>
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> : </t>
+      <t>participation au renouvellement du parc informatique sur le site, avec préparation, masterisation, installation et remplacement de postes de travail et d’écrans. Prise en compte de l’environnement technique local, vérification du bon fonctionnement du matériel et accompagnement des utilisateurs lors de la remise en service.</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>participation à la préparation et à l’accompagnement des utilisateurs dans le cadre de la migration des postes de travail vers Windows 11. Vérification de la compatibilité, assistance aux utilisateurs, résolution des incidents post-migration et suivi des opérations.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>Réorganisation du kiosque IT</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> : </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>participation à la réorganisation du kiosque informatique afin d’améliorer la gestion des équipements, la lisibilité des ressources disponibles et l’efficacité de la prise en charge des utilisateurs.</t>
-    </r>
-  </si>
-  <si>
-    <t>01/04/2025 au 15/04/2025</t>
-  </si>
-  <si>
-    <t>02/09/2024 au 02/09/2024</t>
-  </si>
-  <si>
-    <t>2024-2026</t>
-  </si>
-  <si>
-    <t>2025-2026</t>
+  </si>
+  <si>
+    <t>28/10/2025 au 31/10/2025</t>
+  </si>
+  <si>
+    <t>30/03/2026 au 02/04/2026</t>
   </si>
   <si>
     <r>
@@ -305,7 +364,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>préparation, masterisation, déploiement, renouvellement et maintenance des postes de travail et équipements utilisateurs (PC, iPad, iPhone, imprimantes, Surface Hub). Prise en charge du support utilisateurs de niveau 1 et 2, diagnostic et résolution d’incidents, gestion des comptes et des accès, accompagnement des utilisateurs et rédaction de procédures internes.</t>
+      <t>préparation, masterisation, déploiement, renouvellement et maintenance des postes de travail et équipements utilisateurs (PC, iPad, iPhone, imprimantes, Surface Hub). Prise en charge du support utilisateurs de niveau 1 et 2, diagnostic et résolution d’incidents, gestion des comptes, accompagnement des utilisateurs et rédaction de procédures internes.</t>
     </r>
   </si>
 </sst>
@@ -785,7 +844,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -847,9 +906,58 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -873,54 +981,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1230,7 +1290,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AQ83"/>
+  <dimension ref="A1:AQ82"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="70.44140625" style="1" customWidth="1"/>
@@ -1241,84 +1301,85 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="21"/>
-      <c r="D1" s="21"/>
-      <c r="E1" s="21"/>
-      <c r="F1" s="21"/>
-      <c r="G1" s="21" t="s">
-        <v>23</v>
-      </c>
-      <c r="H1" s="21"/>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27" t="s">
+        <v>38</v>
+      </c>
+      <c r="H1" s="27"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="23"/>
-      <c r="C3" s="23"/>
-      <c r="D3" s="23"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="28" t="s">
-        <v>19</v>
-      </c>
-      <c r="G3" s="23"/>
-      <c r="H3" s="29"/>
+      <c r="A3" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="45" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="40"/>
+      <c r="H3" s="46"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="25" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="27"/>
+      <c r="A4" s="42" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="44"/>
       <c r="F4" s="14" t="s">
         <v>8</v>
       </c>
       <c r="G4" s="15" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="H4" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="I4" s="24"/>
+    </row>
+    <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="36" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38"/>
+    </row>
+    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="25" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="40" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="41"/>
-      <c r="C5" s="41"/>
-      <c r="D5" s="41"/>
-      <c r="E5" s="41"/>
-      <c r="F5" s="41"/>
-      <c r="G5" s="41"/>
-      <c r="H5" s="42"/>
-    </row>
-    <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="30" t="s">
+      <c r="B6" s="34" t="s">
         <v>18</v>
-      </c>
-      <c r="B6" s="38" t="s">
-        <v>20</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>0</v>
@@ -1340,8 +1401,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="31"/>
-      <c r="B7" s="39"/>
+      <c r="A7" s="26"/>
+      <c r="B7" s="35"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1397,16 +1458,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="32" t="s">
-        <v>17</v>
-      </c>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="34"/>
+      <c r="A8" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1445,25 +1506,21 @@
     </row>
     <row r="9" spans="1:43" s="2" customFormat="1" ht="86.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C9" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="G9" s="44" t="s">
-        <v>27</v>
+        <v>29</v>
+      </c>
+      <c r="C9" s="17"/>
+      <c r="D9" s="17"/>
+      <c r="E9" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="G9" s="22" t="s">
+        <v>24</v>
       </c>
       <c r="H9" s="17"/>
       <c r="I9"/>
@@ -1504,25 +1561,19 @@
     </row>
     <row r="10" spans="1:43" s="2" customFormat="1" ht="76.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="C10" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="E10" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="G10" s="44" t="s">
-        <v>27</v>
+      <c r="C10" s="17"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="G10" s="22" t="s">
+        <v>24</v>
       </c>
       <c r="H10" s="17"/>
       <c r="I10"/>
@@ -1563,24 +1614,22 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="76.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>30</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>38</v>
       </c>
       <c r="C11" s="17"/>
       <c r="D11" s="17"/>
-      <c r="E11" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="F11" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="G11" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="H11" s="44" t="s">
-        <v>27</v>
+      <c r="E11" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="G11" s="17"/>
+      <c r="H11" s="22" t="s">
+        <v>24</v>
       </c>
       <c r="I11"/>
       <c r="J11"/>
@@ -1620,22 +1669,20 @@
     </row>
     <row r="12" spans="1:43" s="2" customFormat="1" ht="78" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="C12" s="17"/>
       <c r="D12" s="16"/>
-      <c r="E12" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="44" t="s">
-        <v>27</v>
-      </c>
-      <c r="G12" s="44" t="s">
-        <v>27</v>
-      </c>
+      <c r="E12" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="22" t="s">
+        <v>24</v>
+      </c>
+      <c r="G12" s="17"/>
       <c r="H12" s="17"/>
       <c r="I12"/>
       <c r="J12"/>
@@ -2034,16 +2081,16 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A21" s="35" t="s">
-        <v>21</v>
-      </c>
-      <c r="B21" s="36"/>
-      <c r="C21" s="36"/>
-      <c r="D21" s="36"/>
-      <c r="E21" s="36"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="37"/>
+      <c r="A21" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="32"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="33"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -2082,21 +2129,21 @@
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="115.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C22" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="D22" s="45" t="s">
-        <v>27</v>
+        <v>31</v>
+      </c>
+      <c r="C22" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="D22" s="23" t="s">
+        <v>24</v>
       </c>
       <c r="E22" s="17"/>
       <c r="F22" s="17"/>
-      <c r="G22" s="45" t="s">
-        <v>27</v>
+      <c r="G22" s="23" t="s">
+        <v>24</v>
       </c>
       <c r="H22" s="17"/>
       <c r="I22"/>
@@ -2137,21 +2184,23 @@
     </row>
     <row r="23" spans="1:43" s="2" customFormat="1" ht="116.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B23" s="10"/>
-      <c r="C23" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="D23" s="45" t="s">
-        <v>27</v>
+        <v>25</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="C23" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="D23" s="23" t="s">
+        <v>24</v>
       </c>
       <c r="E23" s="17"/>
-      <c r="F23" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="G23" s="45" t="s">
-        <v>27</v>
+      <c r="F23" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="G23" s="23" t="s">
+        <v>24</v>
       </c>
       <c r="H23" s="17"/>
       <c r="I23"/>
@@ -2192,22 +2241,22 @@
     </row>
     <row r="24" spans="1:43" s="2" customFormat="1" ht="115.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="B24" s="10"/>
-      <c r="C24" s="45" t="s">
         <v>27</v>
       </c>
-      <c r="D24" s="45" t="s">
-        <v>27</v>
+      <c r="B24" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="C24" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24" s="23" t="s">
+        <v>24</v>
       </c>
       <c r="E24" s="17"/>
-      <c r="F24" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="G24" s="45" t="s">
-        <v>27</v>
-      </c>
+      <c r="F24" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="G24" s="17"/>
       <c r="H24" s="17"/>
       <c r="I24"/>
       <c r="J24"/>
@@ -2245,25 +2294,25 @@
       <c r="AP24"/>
       <c r="AQ24"/>
     </row>
-    <row r="25" spans="1:43" s="2" customFormat="1" ht="78.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:43" s="2" customFormat="1" ht="114.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>34</v>
-      </c>
-      <c r="B25" s="43" t="s">
-        <v>35</v>
-      </c>
-      <c r="C25" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="D25" s="45" t="s">
-        <v>27</v>
+        <v>40</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C25" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="D25" s="23" t="s">
+        <v>24</v>
       </c>
       <c r="E25" s="17"/>
-      <c r="F25" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="G25" s="45" t="s">
-        <v>27</v>
+      <c r="F25" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="G25" s="23" t="s">
+        <v>24</v>
       </c>
       <c r="H25" s="17"/>
       <c r="I25"/>
@@ -2306,9 +2355,9 @@
       <c r="A26" s="11"/>
       <c r="B26" s="10"/>
       <c r="C26" s="17"/>
-      <c r="D26" s="20"/>
+      <c r="D26" s="17"/>
       <c r="E26" s="17"/>
-      <c r="F26" s="17"/>
+      <c r="F26" s="20"/>
       <c r="G26" s="17"/>
       <c r="H26" s="17"/>
       <c r="I26"/>
@@ -2353,8 +2402,8 @@
       <c r="C27" s="17"/>
       <c r="D27" s="17"/>
       <c r="E27" s="17"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="17"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="20"/>
       <c r="H27" s="17"/>
       <c r="I27"/>
       <c r="J27"/>
@@ -2392,15 +2441,17 @@
       <c r="AP27"/>
       <c r="AQ27"/>
     </row>
-    <row r="28" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="11"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="17"/>
-      <c r="D28" s="17"/>
-      <c r="E28" s="17"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="17"/>
+    <row r="28" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
+      <c r="A28" s="31" t="s">
+        <v>20</v>
+      </c>
+      <c r="B28" s="32"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="33"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2437,17 +2488,25 @@
       <c r="AP28"/>
       <c r="AQ28"/>
     </row>
-    <row r="29" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A29" s="35" t="s">
-        <v>22</v>
-      </c>
-      <c r="B29" s="36"/>
-      <c r="C29" s="36"/>
-      <c r="D29" s="36"/>
-      <c r="E29" s="36"/>
-      <c r="F29" s="36"/>
-      <c r="G29" s="36"/>
-      <c r="H29" s="37"/>
+    <row r="29" spans="1:43" s="2" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="C29" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="D29" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="H29" s="17"/>
       <c r="I29"/>
       <c r="J29"/>
       <c r="K29"/>
@@ -2484,23 +2543,23 @@
       <c r="AP29"/>
       <c r="AQ29"/>
     </row>
-    <row r="30" spans="1:43" s="2" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:43" s="2" customFormat="1" ht="118.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C30" s="45" t="s">
-        <v>27</v>
-      </c>
-      <c r="D30" s="45" t="s">
-        <v>27</v>
+        <v>26</v>
+      </c>
+      <c r="B30" s="10"/>
+      <c r="C30" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="D30" s="23" t="s">
+        <v>24</v>
       </c>
       <c r="E30" s="17"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="45" t="s">
-        <v>27</v>
+      <c r="F30" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="G30" s="23" t="s">
+        <v>24</v>
       </c>
       <c r="H30" s="17"/>
       <c r="I30"/>
@@ -2539,14 +2598,26 @@
       <c r="AP30"/>
       <c r="AQ30"/>
     </row>
-    <row r="31" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="11"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="17"/>
-      <c r="D31" s="17"/>
+    <row r="31" spans="1:43" s="2" customFormat="1" ht="118.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B31" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="C31" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="D31" s="23" t="s">
+        <v>24</v>
+      </c>
       <c r="E31" s="17"/>
-      <c r="F31" s="17"/>
-      <c r="G31" s="17"/>
+      <c r="F31" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="G31" s="23" t="s">
+        <v>24</v>
+      </c>
       <c r="H31" s="17"/>
       <c r="I31"/>
       <c r="J31"/>
@@ -2719,15 +2790,15 @@
       <c r="AP34"/>
       <c r="AQ34"/>
     </row>
-    <row r="35" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="11"/>
-      <c r="B35" s="10"/>
-      <c r="C35" s="17"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="17"/>
-      <c r="G35" s="17"/>
-      <c r="H35" s="17"/>
+    <row r="35" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="12"/>
+      <c r="B35" s="13"/>
+      <c r="C35" s="18"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="18"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="18"/>
       <c r="I35"/>
       <c r="J35"/>
       <c r="K35"/>
@@ -2764,15 +2835,15 @@
       <c r="AP35"/>
       <c r="AQ35"/>
     </row>
-    <row r="36" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="12"/>
-      <c r="B36" s="13"/>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="18"/>
-      <c r="G36" s="18"/>
-      <c r="H36" s="18"/>
+    <row r="36" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
+      <c r="A36" s="5"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4"/>
       <c r="I36"/>
       <c r="J36"/>
       <c r="K36"/>
@@ -2809,51 +2880,7 @@
       <c r="AP36"/>
       <c r="AQ36"/>
     </row>
-    <row r="37" spans="1:43" s="2" customFormat="1" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A37" s="5"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="4"/>
-      <c r="D37" s="4"/>
-      <c r="E37" s="4"/>
-      <c r="F37" s="4"/>
-      <c r="G37" s="4"/>
-      <c r="H37" s="4"/>
-      <c r="I37"/>
-      <c r="J37"/>
-      <c r="K37"/>
-      <c r="L37"/>
-      <c r="M37"/>
-      <c r="N37"/>
-      <c r="O37"/>
-      <c r="P37"/>
-      <c r="Q37"/>
-      <c r="R37"/>
-      <c r="S37"/>
-      <c r="T37"/>
-      <c r="U37"/>
-      <c r="V37"/>
-      <c r="W37"/>
-      <c r="X37"/>
-      <c r="Y37"/>
-      <c r="Z37"/>
-      <c r="AA37"/>
-      <c r="AB37"/>
-      <c r="AC37"/>
-      <c r="AD37"/>
-      <c r="AE37"/>
-      <c r="AF37"/>
-      <c r="AG37"/>
-      <c r="AH37"/>
-      <c r="AI37"/>
-      <c r="AJ37"/>
-      <c r="AK37"/>
-      <c r="AL37"/>
-      <c r="AM37"/>
-      <c r="AN37"/>
-      <c r="AO37"/>
-      <c r="AP37"/>
-      <c r="AQ37"/>
-    </row>
+    <row r="37" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="38" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="39" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="40" spans="1:43" customFormat="1" x14ac:dyDescent="0.25"/>
@@ -2899,26 +2926,25 @@
     <row r="80" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="82" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="83" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A29:H29"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="A5:H5"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:E3"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="F3:H3"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="A5:H5"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.19685039370078741" right="0.19685039370078741" top="0.19685039370078741" bottom="0.19685039370078741" header="0.51181102362204722" footer="0.51181102362204722"/>
-  <pageSetup paperSize="9" scale="48" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="36" orientation="portrait" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: mettre à jour le lien vers le tableau de synthèse E5 et corriger le contenu des documents
</commit_message>
<xml_diff>
--- a/documents/Tableau_synthese_E5.xlsx
+++ b/documents/Tableau_synthese_E5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Portfolio\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F881C9B3-3619-4FD8-9037-06562F2E2EC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B33E90-E3DA-42A3-BCCC-7D5BE8E116AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -364,7 +364,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>préparation, masterisation, déploiement, renouvellement et maintenance des postes de travail et équipements utilisateurs (PC, iPad, iPhone, imprimantes, Surface Hub). Prise en charge du support utilisateurs de niveau 1 et 2, diagnostic et résolution d’incidents, gestion des comptes, accompagnement des utilisateurs et rédaction de procédures internes.</t>
+      <t>préparation, masterisation, déploiement, renouvellement et maintenance des postes de travail et équipements utilisateurs (PC, iPad, iPhone, imprimantes, Surface Hub). Prise en charge du support utilisateurs de niveau 1 et 2, diagnostic et résolution d’incidents/demandes, gestion des comptes, accompagnement des utilisateurs et rédaction de procédures internes.</t>
     </r>
   </si>
 </sst>
@@ -916,15 +916,39 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -956,30 +980,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1301,56 +1301,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27" t="s">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="H1" s="27"/>
+      <c r="H1" s="25"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="45" t="s">
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="40"/>
-      <c r="H3" s="46"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="33"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="43"/>
-      <c r="C4" s="43"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="44"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="31"/>
       <c r="F4" s="14" t="s">
         <v>8</v>
       </c>
@@ -1363,22 +1363,22 @@
       <c r="I4" s="24"/>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="38"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="46"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="42" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1401,8 +1401,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="26"/>
-      <c r="B7" s="35"/>
+      <c r="A7" s="35"/>
+      <c r="B7" s="43"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1458,16 +1458,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="30"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="38"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -2081,16 +2081,16 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A21" s="31" t="s">
+      <c r="A21" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="32"/>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32"/>
-      <c r="H21" s="33"/>
+      <c r="B21" s="40"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="40"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="41"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -2442,16 +2442,16 @@
       <c r="AQ27"/>
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A28" s="31" t="s">
+      <c r="A28" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="B28" s="32"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="33"/>
+      <c r="B28" s="40"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="40"/>
+      <c r="E28" s="40"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="40"/>
+      <c r="H28" s="41"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2928,11 +2928,6 @@
     <row r="82" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2940,6 +2935,11 @@
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>

<commit_message>
fix: corriger la mise en forme et améliorer la sécurité des requêtes SQL dans le document veille technologique
</commit_message>
<xml_diff>
--- a/documents/Tableau_synthese_E5.xlsx
+++ b/documents/Tableau_synthese_E5.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Portfolio\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00B33E90-E3DA-42A3-BCCC-7D5BE8E116AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDF3E13F-E372-47AD-8A43-6E3582A92AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="45">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -916,9 +916,48 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -941,45 +980,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1301,56 +1301,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25" t="s">
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="H1" s="25"/>
+      <c r="H1" s="27"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="25"/>
-      <c r="C2" s="25"/>
-      <c r="D2" s="25"/>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25"/>
-      <c r="G2" s="25"/>
-      <c r="H2" s="25"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="39" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="27"/>
-      <c r="C3" s="27"/>
-      <c r="D3" s="27"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="32" t="s">
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="45" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="27"/>
-      <c r="H3" s="33"/>
+      <c r="G3" s="40"/>
+      <c r="H3" s="46"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="29" t="s">
+      <c r="A4" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="30"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="31"/>
+      <c r="B4" s="43"/>
+      <c r="C4" s="43"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="44"/>
       <c r="F4" s="14" t="s">
         <v>8</v>
       </c>
@@ -1363,22 +1363,22 @@
       <c r="I4" s="24"/>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="44" t="s">
+      <c r="A5" s="36" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="45"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="46"/>
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="37"/>
+      <c r="E5" s="37"/>
+      <c r="F5" s="37"/>
+      <c r="G5" s="37"/>
+      <c r="H5" s="38"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="42" t="s">
+      <c r="B6" s="34" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1401,8 +1401,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="35"/>
-      <c r="B7" s="43"/>
+      <c r="A7" s="26"/>
+      <c r="B7" s="35"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1458,16 +1458,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="37"/>
-      <c r="C8" s="37"/>
-      <c r="D8" s="37"/>
-      <c r="E8" s="37"/>
-      <c r="F8" s="37"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="38"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="29"/>
+      <c r="D8" s="29"/>
+      <c r="E8" s="29"/>
+      <c r="F8" s="29"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="30"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1566,7 +1566,9 @@
       <c r="B10" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="17"/>
+      <c r="C10" s="22" t="s">
+        <v>24</v>
+      </c>
       <c r="D10" s="17"/>
       <c r="E10" s="17"/>
       <c r="F10" s="22" t="s">
@@ -2081,16 +2083,16 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A21" s="39" t="s">
+      <c r="A21" s="31" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="40"/>
-      <c r="C21" s="40"/>
-      <c r="D21" s="40"/>
-      <c r="E21" s="40"/>
-      <c r="F21" s="40"/>
-      <c r="G21" s="40"/>
-      <c r="H21" s="41"/>
+      <c r="B21" s="32"/>
+      <c r="C21" s="32"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="32"/>
+      <c r="F21" s="32"/>
+      <c r="G21" s="32"/>
+      <c r="H21" s="33"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -2442,16 +2444,16 @@
       <c r="AQ27"/>
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A28" s="39" t="s">
+      <c r="A28" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="B28" s="40"/>
-      <c r="C28" s="40"/>
-      <c r="D28" s="40"/>
-      <c r="E28" s="40"/>
-      <c r="F28" s="40"/>
-      <c r="G28" s="40"/>
-      <c r="H28" s="41"/>
+      <c r="B28" s="32"/>
+      <c r="C28" s="32"/>
+      <c r="D28" s="32"/>
+      <c r="E28" s="32"/>
+      <c r="F28" s="32"/>
+      <c r="G28" s="32"/>
+      <c r="H28" s="33"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2928,6 +2930,11 @@
     <row r="82" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2935,11 +2942,6 @@
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>

<commit_message>
fix: corriger la mise en forme et mettre à jour les dates dans le tableau de synthèse E5
</commit_message>
<xml_diff>
--- a/documents/Tableau_synthese_E5.xlsx
+++ b/documents/Tableau_synthese_E5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\Portfolio\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDF3E13F-E372-47AD-8A43-6E3582A92AB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB4D0BC8-E938-4599-AF43-C26B1393DE36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="44">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -318,9 +318,6 @@
   </si>
   <si>
     <t>SESSION 2026</t>
-  </si>
-  <si>
-    <t>02/09/2024 au …</t>
   </si>
   <si>
     <r>
@@ -916,15 +913,39 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -956,30 +977,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1301,56 +1298,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="27" t="s">
+      <c r="A1" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27" t="s">
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25" t="s">
         <v>38</v>
       </c>
-      <c r="H1" s="27"/>
+      <c r="H1" s="25"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
+      <c r="B2" s="25"/>
+      <c r="C2" s="25"/>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+      <c r="H2" s="25"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="40"/>
-      <c r="C3" s="40"/>
-      <c r="D3" s="40"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="45" t="s">
+      <c r="B3" s="27"/>
+      <c r="C3" s="27"/>
+      <c r="D3" s="27"/>
+      <c r="E3" s="28"/>
+      <c r="F3" s="32" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="40"/>
-      <c r="H3" s="46"/>
+      <c r="G3" s="27"/>
+      <c r="H3" s="33"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="42" t="s">
+      <c r="A4" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="B4" s="43"/>
-      <c r="C4" s="43"/>
-      <c r="D4" s="43"/>
-      <c r="E4" s="44"/>
+      <c r="B4" s="30"/>
+      <c r="C4" s="30"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="31"/>
       <c r="F4" s="14" t="s">
         <v>8</v>
       </c>
@@ -1363,22 +1360,22 @@
       <c r="I4" s="24"/>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="37"/>
-      <c r="D5" s="37"/>
-      <c r="E5" s="37"/>
-      <c r="F5" s="37"/>
-      <c r="G5" s="37"/>
-      <c r="H5" s="38"/>
+      <c r="B5" s="45"/>
+      <c r="C5" s="45"/>
+      <c r="D5" s="45"/>
+      <c r="E5" s="45"/>
+      <c r="F5" s="45"/>
+      <c r="G5" s="45"/>
+      <c r="H5" s="46"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="25" t="s">
+      <c r="A6" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="34" t="s">
+      <c r="B6" s="42" t="s">
         <v>18</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1401,8 +1398,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="26"/>
-      <c r="B7" s="35"/>
+      <c r="A7" s="35"/>
+      <c r="B7" s="43"/>
       <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
@@ -1458,16 +1455,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A8" s="28" t="s">
+      <c r="A8" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="29"/>
-      <c r="C8" s="29"/>
-      <c r="D8" s="29"/>
-      <c r="E8" s="29"/>
-      <c r="F8" s="29"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="30"/>
+      <c r="B8" s="37"/>
+      <c r="C8" s="37"/>
+      <c r="D8" s="37"/>
+      <c r="E8" s="37"/>
+      <c r="F8" s="37"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="38"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -2083,16 +2080,16 @@
       <c r="AQ20"/>
     </row>
     <row r="21" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A21" s="31" t="s">
+      <c r="A21" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="32"/>
-      <c r="C21" s="32"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="32"/>
-      <c r="F21" s="32"/>
-      <c r="G21" s="32"/>
-      <c r="H21" s="33"/>
+      <c r="B21" s="40"/>
+      <c r="C21" s="40"/>
+      <c r="D21" s="40"/>
+      <c r="E21" s="40"/>
+      <c r="F21" s="40"/>
+      <c r="G21" s="40"/>
+      <c r="H21" s="41"/>
       <c r="I21"/>
       <c r="J21"/>
       <c r="K21"/>
@@ -2131,7 +2128,7 @@
     </row>
     <row r="22" spans="1:43" s="2" customFormat="1" ht="115.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B22" s="10" t="s">
         <v>31</v>
@@ -2189,7 +2186,7 @@
         <v>25</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="C23" s="23" t="s">
         <v>24</v>
@@ -2298,10 +2295,10 @@
     </row>
     <row r="25" spans="1:43" s="2" customFormat="1" ht="114.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C25" s="23" t="s">
         <v>24</v>
@@ -2444,16 +2441,16 @@
       <c r="AQ27"/>
     </row>
     <row r="28" spans="1:43" s="2" customFormat="1" ht="17.399999999999999" x14ac:dyDescent="0.25">
-      <c r="A28" s="31" t="s">
+      <c r="A28" s="39" t="s">
         <v>20</v>
       </c>
-      <c r="B28" s="32"/>
-      <c r="C28" s="32"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="32"/>
-      <c r="F28" s="32"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="33"/>
+      <c r="B28" s="40"/>
+      <c r="C28" s="40"/>
+      <c r="D28" s="40"/>
+      <c r="E28" s="40"/>
+      <c r="F28" s="40"/>
+      <c r="G28" s="40"/>
+      <c r="H28" s="41"/>
       <c r="I28"/>
       <c r="J28"/>
       <c r="K28"/>
@@ -2492,7 +2489,7 @@
     </row>
     <row r="29" spans="1:43" s="2" customFormat="1" ht="117" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="11" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B29" s="10" t="s">
         <v>31</v>
@@ -2602,10 +2599,10 @@
     </row>
     <row r="31" spans="1:43" s="2" customFormat="1" ht="118.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C31" s="23" t="s">
         <v>24</v>
@@ -2930,11 +2927,6 @@
     <row r="82" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2942,6 +2934,11 @@
     <mergeCell ref="A28:H28"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>